<commit_message>
Adjusted BPT diagrams and began adding high-z galaxies to plots
</commit_message>
<xml_diff>
--- a/CLASSY/Final_CLASSY_EMISSION_LINES_David.xlsx
+++ b/CLASSY/Final_CLASSY_EMISSION_LINES_David.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0013ccd3bb406478/Senior Honours Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0013ccd3bb406478/Senior Honours Project/CLASSY/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{6A61F873-5642-1F4E-9EEC-E5CE1B3A1FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B7BFCD2-0602-4E16-A653-7F87CAD24FDE}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{6A61F873-5642-1F4E-9EEC-E5CE1B3A1FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9015C607-DFF2-40FF-8FFB-B926460CB849}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{61282016-CF89-B44E-B0FA-48962238AFD8}"/>
   </bookViews>
@@ -237,9 +237,6 @@
   </si>
   <si>
     <t>SN_ha</t>
-  </si>
-  <si>
-    <t>nii6584</t>
   </si>
   <si>
     <t>EUP_nii6584</t>
@@ -472,6 +469,9 @@
   <si>
     <t>SN_neiii3870</t>
   </si>
+  <si>
+    <t>F</t>
+  </si>
 </sst>
 </file>
 
@@ -558,10 +558,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1101,105 +1097,105 @@
         <v>66</v>
       </c>
       <c r="BP1" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="BQ1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="BQ1" s="1" t="s">
+      <c r="BR1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="BR1" s="1" t="s">
+      <c r="BS1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="BS1" s="1" t="s">
+      <c r="BT1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="BT1" s="1" t="s">
+      <c r="BU1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="BU1" s="1" t="s">
+      <c r="BV1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="BV1" s="1" t="s">
+      <c r="BW1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="BW1" s="1" t="s">
+      <c r="BX1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="BX1" s="1" t="s">
+      <c r="BY1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="BY1" s="1" t="s">
+      <c r="BZ1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="BZ1" s="1" t="s">
+      <c r="CA1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="CA1" s="1" t="s">
+      <c r="CB1" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="CB1" s="5" t="s">
+      <c r="CC1" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="CC1" s="5" t="s">
+      <c r="CD1" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="CD1" s="5" t="s">
+      <c r="CE1" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="CE1" s="5" t="s">
+      <c r="CF1" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="CF1" s="5" t="s">
+      <c r="CG1" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="CG1" s="5" t="s">
+      <c r="CH1" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="CH1" s="5" t="s">
+      <c r="CI1" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="CI1" s="5" t="s">
+      <c r="CJ1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="CJ1" s="1" t="s">
+      <c r="CK1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="CK1" s="1" t="s">
+      <c r="CL1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="CL1" s="1" t="s">
+      <c r="CM1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="CM1" s="1" t="s">
+      <c r="CN1" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="CN1" s="4" t="s">
+      <c r="CO1" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="CO1" s="4" t="s">
+      <c r="CP1" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="CP1" s="4" t="s">
+      <c r="CQ1" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="CQ1" s="4" t="s">
-        <v>94</v>
-      </c>
       <c r="CR1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="CS1" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="CS1" s="1" t="s">
+      <c r="CT1" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="CT1" s="1" t="s">
+      <c r="CU1" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="CU1" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="2" spans="1:99">
       <c r="A2" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B2" s="5">
         <v>51.352590101392501</v>
@@ -1286,10 +1282,10 @@
         <v>34.435154781732798</v>
       </c>
       <c r="AD2" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AE2" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AF2" s="1">
         <v>0.23783369449642</v>
@@ -1472,16 +1468,16 @@
         <v>390.85815070347797</v>
       </c>
       <c r="CN2" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO2" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP2" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ2" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR2" s="1">
         <v>19.8260311711445</v>
@@ -1498,67 +1494,67 @@
     </row>
     <row r="3" spans="1:99">
       <c r="A3" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="V3" s="1">
         <v>1.8802363500447501</v>
@@ -1783,57 +1779,57 @@
         <v>2320.87084029687</v>
       </c>
       <c r="CR3" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CS3" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CT3" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CU3" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:99">
       <c r="A4" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="N4" s="1">
         <v>1041.79895612214</v>
@@ -1860,28 +1856,28 @@
         <v>27.606877015107099</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="W4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="X4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="Y4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AB4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AC4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AD4" s="1">
         <v>27.8114166980634</v>
@@ -1890,28 +1886,28 @@
         <v>11.182240106834399</v>
       </c>
       <c r="AF4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AG4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AH4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AI4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AJ4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AK4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AL4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AM4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AN4" s="1">
         <v>2197.3168016222899</v>
@@ -2070,33 +2066,33 @@
         <v>75.390324097783505</v>
       </c>
       <c r="CN4" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO4" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP4" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ4" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CS4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CT4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CU4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:99">
       <c r="A5" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B5" s="5">
         <v>16.228669492647601</v>
@@ -2123,28 +2119,28 @@
         <v>7.7856134588521302</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="R5" s="2">
         <v>1.60320532121407</v>
@@ -2249,16 +2245,16 @@
         <v>4.7007145525447198</v>
       </c>
       <c r="AZ5" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BA5" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BB5" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BC5" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BD5" s="1">
         <v>0.47900527074312699</v>
@@ -2333,129 +2329,129 @@
         <v>4.65394020591103</v>
       </c>
       <c r="CB5" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CC5" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CD5" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CE5" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CF5" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CG5" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CH5" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CI5" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CJ5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CK5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CL5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CM5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CN5" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO5" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP5" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ5" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CS5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CT5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CU5" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:99">
       <c r="A6" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="U6" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="V6" s="1">
         <v>2.11356465497891</v>
@@ -2548,16 +2544,16 @@
         <v>3036.76314741135</v>
       </c>
       <c r="AZ6" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BA6" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BB6" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BC6" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BD6" s="1">
         <v>0.317061913258882</v>
@@ -2680,81 +2676,81 @@
         <v>482.27908828240498</v>
       </c>
       <c r="CR6" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CS6" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CT6" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CU6" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:99">
       <c r="A7" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="U7" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="V7" s="1">
         <v>0.154231037030786</v>
@@ -2979,21 +2975,21 @@
         <v>49.141202466800699</v>
       </c>
       <c r="CR7" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CS7" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CT7" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CU7" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:99">
       <c r="A8" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B8" s="5">
         <v>5.9736596130008</v>
@@ -3044,28 +3040,28 @@
         <v>55.204295068752899</v>
       </c>
       <c r="R8" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="S8" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="U8" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="X8" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="Y8" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="Z8" s="1">
         <v>0.32034841025701799</v>
@@ -3134,13 +3130,13 @@
         <v>28.057229194213601</v>
       </c>
       <c r="AV8" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AW8" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AX8" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AY8" s="1">
         <v>61.651938038648503</v>
@@ -3158,28 +3154,28 @@
         <v>19.990257496094799</v>
       </c>
       <c r="BD8" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BE8" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BF8" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BG8" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BH8" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BI8" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BJ8" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BK8" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BL8" s="1">
         <v>32.183383564721403</v>
@@ -3292,7 +3288,7 @@
     </row>
     <row r="9" spans="1:99">
       <c r="A9" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B9" s="5">
         <v>130.24510669967299</v>
@@ -3565,16 +3561,16 @@
         <v>116.191636295775</v>
       </c>
       <c r="CN9" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO9" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP9" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ9" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR9" s="1">
         <v>44.173100451520703</v>
@@ -3591,7 +3587,7 @@
     </row>
     <row r="10" spans="1:99">
       <c r="A10" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B10" s="5">
         <v>11.5938322791399</v>
@@ -3864,16 +3860,16 @@
         <v>23.659297995525701</v>
       </c>
       <c r="CN10" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO10" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP10" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ10" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR10" s="1">
         <v>6.78018119829136</v>
@@ -3890,7 +3886,7 @@
     </row>
     <row r="11" spans="1:99">
       <c r="A11" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B11" s="5">
         <v>2.3374542147698101</v>
@@ -4043,153 +4039,153 @@
         <v>770.58883194447503</v>
       </c>
       <c r="AZ11" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BA11" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BB11" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BC11" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BD11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BE11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BF11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BG11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BH11" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BI11" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BJ11" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BK11" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BL11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BM11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BN11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BO11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BP11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BQ11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BR11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BS11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BT11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BU11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BV11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BW11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BX11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BY11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BZ11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CA11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CB11" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CC11" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CD11" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CE11" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CF11" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CG11" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CH11" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CI11" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CJ11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CK11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CL11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CM11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CN11" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO11" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP11" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ11" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CS11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CT11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CU11" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" spans="1:99">
       <c r="A12" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B12" s="5">
         <v>34.04596526225</v>
@@ -4462,16 +4458,16 @@
         <v>59.339320289748997</v>
       </c>
       <c r="CN12" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO12" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP12" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ12" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR12" s="1">
         <v>11.400524224247</v>
@@ -4488,31 +4484,31 @@
     </row>
     <row r="13" spans="1:99">
       <c r="A13" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J13" s="1">
         <v>1.9207945131418001</v>
@@ -4787,31 +4783,31 @@
     </row>
     <row r="14" spans="1:99">
       <c r="A14" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J14" s="1">
         <v>8.4733168193072093</v>
@@ -5060,13 +5056,13 @@
         <v>47.819242886798499</v>
       </c>
       <c r="CN14" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO14" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP14" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ14" s="4">
         <v>0.71766908678116803</v>
@@ -5086,19 +5082,19 @@
     </row>
     <row r="15" spans="1:99">
       <c r="A15" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F15" s="5">
         <v>3261201.1723690098</v>
@@ -5239,16 +5235,16 @@
         <v>112.775458829252</v>
       </c>
       <c r="AZ15" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BA15" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BB15" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BC15" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BD15" s="1">
         <v>0.329903534980307</v>
@@ -5359,16 +5355,16 @@
         <v>4.5708241915016004</v>
       </c>
       <c r="CN15" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO15" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP15" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ15" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR15" s="1">
         <v>1.03972367358637</v>
@@ -5385,7 +5381,7 @@
     </row>
     <row r="16" spans="1:99">
       <c r="A16" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B16" s="5">
         <v>6.4018981083198403</v>
@@ -5622,28 +5618,28 @@
         <v>654.42893281020201</v>
       </c>
       <c r="CB16" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CC16" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CD16" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CE16" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CF16" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CG16" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CH16" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CI16" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CJ16" s="1">
         <v>1.4945080260255399</v>
@@ -5684,31 +5680,31 @@
     </row>
     <row r="17" spans="1:99">
       <c r="A17" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J17" s="1">
         <v>17.6155701374778</v>
@@ -5983,7 +5979,7 @@
     </row>
     <row r="18" spans="1:99">
       <c r="A18" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B18" s="5">
         <v>31.3520741700668</v>
@@ -6256,16 +6252,16 @@
         <v>66.3770350070305</v>
       </c>
       <c r="CN18" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO18" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP18" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ18" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR18" s="1">
         <v>19.506613527499201</v>
@@ -6282,7 +6278,7 @@
     </row>
     <row r="19" spans="1:99">
       <c r="A19" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B19" s="5">
         <v>15.2115200413559</v>
@@ -6555,16 +6551,16 @@
         <v>42.484562835329299</v>
       </c>
       <c r="CN19" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO19" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP19" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ19" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR19" s="1">
         <v>6.8707934291211901</v>
@@ -6581,31 +6577,31 @@
     </row>
     <row r="20" spans="1:99">
       <c r="A20" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J20" s="1">
         <v>14.642419106575799</v>
@@ -6734,16 +6730,16 @@
         <v>302.82307469349399</v>
       </c>
       <c r="AZ20" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BA20" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BB20" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BC20" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BD20" s="1">
         <v>0.39915932229996398</v>
@@ -6880,7 +6876,7 @@
     </row>
     <row r="21" spans="1:99">
       <c r="A21" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B21" s="5">
         <v>194.18059781776699</v>
@@ -7153,16 +7149,16 @@
         <v>95.357858344074401</v>
       </c>
       <c r="CN21" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO21" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP21" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ21" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR21" s="1">
         <v>55.988150221726897</v>
@@ -7179,7 +7175,7 @@
     </row>
     <row r="22" spans="1:99">
       <c r="A22" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B22" s="5">
         <v>49.384779670777696</v>
@@ -7452,16 +7448,16 @@
         <v>33.817856177244202</v>
       </c>
       <c r="CN22" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO22" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP22" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ22" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR22" s="1">
         <v>5.5807354802231197</v>
@@ -7478,31 +7474,31 @@
     </row>
     <row r="23" spans="1:99">
       <c r="A23" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J23" s="1">
         <v>4.7095369585298803</v>
@@ -7777,43 +7773,43 @@
     </row>
     <row r="24" spans="1:99">
       <c r="A24" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="N24" s="1">
         <v>37.220360311487603</v>
@@ -8076,7 +8072,7 @@
     </row>
     <row r="25" spans="1:99">
       <c r="A25" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B25" s="5">
         <v>44.999203347223997</v>
@@ -8349,16 +8345,16 @@
         <v>102.452924864574</v>
       </c>
       <c r="CN25" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO25" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP25" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ25" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR25" s="1">
         <v>20.174964411589201</v>
@@ -8375,31 +8371,31 @@
     </row>
     <row r="26" spans="1:99">
       <c r="A26" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J26" s="1">
         <v>3.2705956862124901</v>
@@ -8528,16 +8524,16 @@
         <v>177.115959898287</v>
       </c>
       <c r="AZ26" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BA26" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BB26" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BC26" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BD26" s="1">
         <v>0.45730655926686598</v>
@@ -8674,7 +8670,7 @@
     </row>
     <row r="27" spans="1:99">
       <c r="A27" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B27" s="5">
         <v>21.125022492137699</v>
@@ -8749,16 +8745,16 @@
         <v>3.2933534441583401</v>
       </c>
       <c r="Z27" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AA27" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AB27" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AC27" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AD27" s="1">
         <v>8.7588127678941793E-2</v>
@@ -8767,28 +8763,28 @@
         <v>1.1555698424373599</v>
       </c>
       <c r="AF27" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AG27" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AH27" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AI27" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AJ27" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AK27" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AL27" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AM27" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AN27" s="1">
         <v>11.3279875991126</v>
@@ -8827,16 +8823,16 @@
         <v>83.953605434198593</v>
       </c>
       <c r="AZ27" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BA27" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BB27" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BC27" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BD27" s="1">
         <v>1.0777659562417401</v>
@@ -8947,16 +8943,16 @@
         <v>14.1621088680184</v>
       </c>
       <c r="CN27" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO27" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP27" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ27" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR27" s="1">
         <v>3.0060226820031999</v>
@@ -8973,7 +8969,7 @@
     </row>
     <row r="28" spans="1:99">
       <c r="A28" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B28" s="5">
         <v>4.8518108537585301</v>
@@ -9272,31 +9268,31 @@
     </row>
     <row r="29" spans="1:99">
       <c r="A29" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J29" s="1">
         <v>36.5473130624937</v>
@@ -9571,31 +9567,31 @@
     </row>
     <row r="30" spans="1:99">
       <c r="A30" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J30" s="1">
         <v>28.678212346634499</v>
@@ -9870,7 +9866,7 @@
     </row>
     <row r="31" spans="1:99">
       <c r="A31" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B31" s="5">
         <v>39.24652915891</v>
@@ -10143,16 +10139,16 @@
         <v>57.038256574573602</v>
       </c>
       <c r="CN31" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO31" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP31" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ31" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR31" s="1">
         <v>22.298951968011099</v>
@@ -10169,31 +10165,31 @@
     </row>
     <row r="32" spans="1:99">
       <c r="A32" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J32" s="1">
         <v>31.8624645508805</v>
@@ -10468,7 +10464,7 @@
     </row>
     <row r="33" spans="1:99">
       <c r="A33" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B33" s="5">
         <v>160.927505847791</v>
@@ -10657,13 +10653,13 @@
         <v>69.911497606401497</v>
       </c>
       <c r="BL33" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BM33" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BN33" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BO33" s="1">
         <v>16.930299830273199</v>
@@ -10741,16 +10737,16 @@
         <v>141.14066638641199</v>
       </c>
       <c r="CN33" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO33" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP33" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ33" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR33" s="1">
         <v>165.875176314339</v>
@@ -10767,31 +10763,31 @@
     </row>
     <row r="34" spans="1:99">
       <c r="A34" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J34" s="1">
         <v>38.760325595806002</v>
@@ -11066,7 +11062,7 @@
     </row>
     <row r="35" spans="1:99">
       <c r="A35" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B35" s="5">
         <v>1.2335552289879399</v>
@@ -11365,7 +11361,7 @@
     </row>
     <row r="36" spans="1:99">
       <c r="A36" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B36" s="5">
         <v>52.445091977968403</v>
@@ -11638,16 +11634,16 @@
         <v>60.039385365220497</v>
       </c>
       <c r="CN36" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO36" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP36" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ36" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR36" s="1">
         <v>23.205258098047398</v>
@@ -11664,7 +11660,7 @@
     </row>
     <row r="37" spans="1:99">
       <c r="A37" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B37" s="5">
         <v>50.808646812882799</v>
@@ -11817,16 +11813,16 @@
         <v>93.225685725589898</v>
       </c>
       <c r="AZ37" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BA37" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BB37" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BC37" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BD37" s="1">
         <v>1.72570344181464</v>
@@ -11937,16 +11933,16 @@
         <v>24.4796780710797</v>
       </c>
       <c r="CN37" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO37" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP37" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ37" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR37" s="1">
         <v>6.9431368787636796</v>
@@ -11963,43 +11959,43 @@
     </row>
     <row r="38" spans="1:99">
       <c r="A38" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="N38" s="1">
         <v>21.6083050262684</v>
@@ -12116,16 +12112,16 @@
         <v>250.46871729062201</v>
       </c>
       <c r="AZ38" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BA38" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BB38" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BC38" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BD38" s="1">
         <v>0.585642233458739</v>
@@ -12262,7 +12258,7 @@
     </row>
     <row r="39" spans="1:99">
       <c r="A39" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B39" s="5">
         <v>19.576585431190399</v>
@@ -12367,16 +12363,16 @@
         <v>0.56732566408229501</v>
       </c>
       <c r="AJ39" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AK39" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AL39" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AM39" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AN39" s="1">
         <v>12.803121890485301</v>
@@ -12535,16 +12531,16 @@
         <v>16.4600898643831</v>
       </c>
       <c r="CN39" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO39" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP39" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ39" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR39" s="1">
         <v>4.3306464551606503</v>
@@ -12561,7 +12557,7 @@
     </row>
     <row r="40" spans="1:99">
       <c r="A40" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B40" s="5">
         <v>25.895879609198701</v>
@@ -12834,16 +12830,16 @@
         <v>52.586895123222902</v>
       </c>
       <c r="CN40" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO40" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP40" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ40" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR40" s="1">
         <v>16.790294785403699</v>
@@ -12860,31 +12856,31 @@
     </row>
     <row r="41" spans="1:99">
       <c r="A41" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I41" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J41" s="1">
         <v>0.80958927183263096</v>
@@ -12953,16 +12949,16 @@
         <v>1.3787906369701</v>
       </c>
       <c r="AF41" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AG41" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AH41" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AI41" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AJ41" s="1">
         <v>6.45073397512647E-2</v>
@@ -13159,7 +13155,7 @@
     </row>
     <row r="42" spans="1:99">
       <c r="A42" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B42" s="5">
         <v>49.837552020635897</v>
@@ -13432,16 +13428,16 @@
         <v>111.97376495676301</v>
       </c>
       <c r="CN42" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO42" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP42" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ42" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR42" s="1">
         <v>44.366178247350099</v>
@@ -13458,7 +13454,7 @@
     </row>
     <row r="43" spans="1:99">
       <c r="A43" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B43" s="5">
         <v>25.252546201920101</v>
@@ -13731,16 +13727,16 @@
         <v>22.6165870492019</v>
       </c>
       <c r="CN43" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO43" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP43" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ43" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR43" s="1">
         <v>8.5441405633113607</v>
@@ -13757,7 +13753,7 @@
     </row>
     <row r="44" spans="1:99">
       <c r="A44" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B44" s="5">
         <v>66.675703461812304</v>
@@ -13850,16 +13846,16 @@
         <v>4.4963879381012397</v>
       </c>
       <c r="AF44" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AG44" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AH44" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AI44" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AJ44" s="1">
         <v>0.30469152549532602</v>
@@ -14030,16 +14026,16 @@
         <v>30.4045003455781</v>
       </c>
       <c r="CN44" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO44" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP44" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ44" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR44" s="1">
         <v>7.7106692998807604</v>
@@ -14056,7 +14052,7 @@
     </row>
     <row r="45" spans="1:99">
       <c r="A45" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B45" s="5">
         <v>10.1740211031137</v>
@@ -14209,16 +14205,16 @@
         <v>6317.2730720031795</v>
       </c>
       <c r="AZ45" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BA45" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BB45" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BC45" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BD45" s="1">
         <v>0.66525691710351298</v>
@@ -14293,28 +14289,28 @@
         <v>499.71032874142401</v>
       </c>
       <c r="CB45" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CC45" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CD45" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CE45" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CF45" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CG45" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CH45" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CI45" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CJ45" s="1">
         <v>1.7445815114801599</v>
@@ -14355,7 +14351,7 @@
     </row>
     <row r="46" spans="1:99">
       <c r="A46" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B46" s="5">
         <v>62.559329127580497</v>
@@ -14628,16 +14624,16 @@
         <v>28.9691627190888</v>
       </c>
       <c r="CN46" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CO46" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CP46" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CQ46" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="CR46" s="1">
         <v>7.6258499716215997</v>

</xml_diff>